<commit_message>
Add Gallaudet to the sports art checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AB9Rj1P6bK7dh1whTDXVpZ
</commit_message>
<xml_diff>
--- a/docs/jl-sports-art-checklist.xlsx
+++ b/docs/jl-sports-art-checklist.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$1:$R$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$1:$R$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R64"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6019,8 +6019,610 @@
       </c>
       <c r="R64" s="2" t="inlineStr"/>
     </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>NCAA D-III</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison [SCAC]</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>hero.jpg</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Hero</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>3840×2160</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>JPG or WebP</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Sports page top banner, team page</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Subject on the right half; left 45% calm and darker for text</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>JL Vision (team_slug, no ESPN id needed)</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="N65" s="3" t="inlineStr">
+        <is>
+          <t>not on ESPN</t>
+        </is>
+      </c>
+      <c r="O65" s="3" t="inlineStr">
+        <is>
+          <t>(by team_slug)</t>
+        </is>
+      </c>
+      <c r="P65" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Q65" s="3" t="inlineStr">
+        <is>
+          <t>Original art</t>
+        </is>
+      </c>
+      <c r="R65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>NCAA D-III</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison [SCAC]</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>wordmark.png</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Wordmark</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>~2000 px wide</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Transparent PNG</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Over the hero, replaces the typed name</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Team name in display lettering; must read on dark backgrounds</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>JL Vision (team_slug, no ESPN id needed)</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="M66" s="3" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="N66" s="3" t="inlineStr">
+        <is>
+          <t>not on ESPN</t>
+        </is>
+      </c>
+      <c r="O66" s="3" t="inlineStr">
+        <is>
+          <t>(by team_slug)</t>
+        </is>
+      </c>
+      <c r="P66" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Q66" s="3" t="inlineStr">
+        <is>
+          <t>Original art</t>
+        </is>
+      </c>
+      <c r="R66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>NCAA D-III</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison [SCAC]</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>card.jpg</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>1920×1080</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>JPG or WebP</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Live Sports Channels cards, game cards</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Bottom third darker (scores sit there)</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>JL Vision (team_slug, no ESPN id needed)</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="N67" s="3" t="inlineStr">
+        <is>
+          <t>not on ESPN</t>
+        </is>
+      </c>
+      <c r="O67" s="3" t="inlineStr">
+        <is>
+          <t>(by team_slug)</t>
+        </is>
+      </c>
+      <c r="P67" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Q67" s="3" t="inlineStr">
+        <is>
+          <t>Original art</t>
+        </is>
+      </c>
+      <c r="R67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>NCAA D-III</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison [SCAC]</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>story.jpg</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>1080×1080</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>JPG or WebP</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>Game Stories circles</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Subject centred; cropped to a circle</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>JL Vision (team_slug, no ESPN id needed)</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="N68" s="3" t="inlineStr">
+        <is>
+          <t>not on ESPN</t>
+        </is>
+      </c>
+      <c r="O68" s="3" t="inlineStr">
+        <is>
+          <t>(by team_slug)</t>
+        </is>
+      </c>
+      <c r="P68" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Q68" s="3" t="inlineStr">
+        <is>
+          <t>Original art</t>
+        </is>
+      </c>
+      <c r="R68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>NCAA D-III</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison [SCAC]</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>(no file)</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Team colours</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Hex codes</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Whole hub switches to the team's look</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Fill the Colours sheet; mark verified only when checked against the official guide</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>team_brand_themes (is_verified = true)</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="N69" s="3" t="inlineStr">
+        <is>
+          <t>not on ESPN</t>
+        </is>
+      </c>
+      <c r="O69" s="3" t="inlineStr">
+        <is>
+          <t>(by team_slug)</t>
+        </is>
+      </c>
+      <c r="P69" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Q69" s="3" t="inlineStr">
+        <is>
+          <t>Original art</t>
+        </is>
+      </c>
+      <c r="R69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>NCAA D-III</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison [SCAC]</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>background.jpg</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Clean background</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>3840×2160</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>JPG or WebP</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>Behind JL Vision templates (hero banner, posters)</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Stadium atmosphere in team colours. NO logos, NO text</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>JL Vision generated_design_assets</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="N70" s="3" t="inlineStr">
+        <is>
+          <t>not on ESPN</t>
+        </is>
+      </c>
+      <c r="O70" s="3" t="inlineStr">
+        <is>
+          <t>(by team_slug)</t>
+        </is>
+      </c>
+      <c r="P70" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Q70" s="3" t="inlineStr">
+        <is>
+          <t>Original art</t>
+        </is>
+      </c>
+      <c r="R70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>NCAA D-III</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison [SCAC]</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>wallpaper.jpg</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Wallpaper</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>3840×2160</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>JPG or WebP</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Pin to wallpaper / page background</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>Quiet and atmospheric; video and menus sit on top</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>JL Vision (team_slug, no ESPN id needed)</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="N71" s="3" t="inlineStr">
+        <is>
+          <t>not on ESPN</t>
+        </is>
+      </c>
+      <c r="O71" s="3" t="inlineStr">
+        <is>
+          <t>(by team_slug)</t>
+        </is>
+      </c>
+      <c r="P71" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="Q71" s="3" t="inlineStr">
+        <is>
+          <t>Original art</t>
+        </is>
+      </c>
+      <c r="R71" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R64"/>
+  <autoFilter ref="A1:R71"/>
   <conditionalFormatting sqref="P2:P64">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Live in app"</formula>
@@ -6041,10 +6643,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="P2:P64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="P2:P71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,In progress,Delivered,Uploaded,Live in app"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Q2:Q71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Original art,Licensed,Needs check"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6058,7 +6660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6183,15 +6785,6 @@
           <t>oregon</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>24</v>
       </c>
@@ -6203,7 +6796,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>No</t>
@@ -6226,15 +6818,6 @@
           <t>ohio-state</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>24</v>
       </c>
@@ -6246,7 +6829,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>No</t>
@@ -6269,15 +6851,6 @@
           <t>alabama</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>24</v>
       </c>
@@ -6289,7 +6862,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>No</t>
@@ -6312,15 +6884,6 @@
           <t>miami-fl</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>24</v>
       </c>
@@ -6332,7 +6895,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
           <t>No</t>
@@ -6355,15 +6917,6 @@
           <t>penn-state</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
         <v>24</v>
       </c>
@@ -6375,7 +6928,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
           <t>No</t>
@@ -6398,15 +6950,6 @@
           <t>seattle-seahawks</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>24</v>
       </c>
@@ -6418,7 +6961,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
           <t>No</t>
@@ -6441,15 +6983,6 @@
           <t>philadelphia-eagles</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
         <v>24</v>
       </c>
@@ -6461,7 +6994,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
           <t>No</t>
@@ -6484,15 +7016,6 @@
           <t>chicago-bears</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
         <v>24</v>
       </c>
@@ -6504,7 +7027,6 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
           <t>No</t>
@@ -6527,15 +7049,6 @@
           <t>detroit-lions</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>24</v>
       </c>
@@ -6547,15 +7060,58 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gallaudet Bison</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>scac</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>gallaudet</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>24</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>glass_ios_vision</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Every colour is #RRGGBB (for example #154733). The app uses a palette only when all nine colours are filled and Verified? is Yes.</t>
         </is>
@@ -6563,10 +7119,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="Q2:Q10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Q2:Q11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O2:O11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"glass_ios_vision,glass_morphism,ios_vision_sports,cinematic_sports,premium_card"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Mark Gallaudet's ESPN id as not linked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AB9Rj1P6bK7dh1whTDXVpZ
</commit_message>
<xml_diff>
--- a/docs/jl-sports-art-checklist.xlsx
+++ b/docs/jl-sports-art-checklist.xlsx
@@ -6085,7 +6085,7 @@
       </c>
       <c r="N65" s="3" t="inlineStr">
         <is>
-          <t>not on ESPN</t>
+          <t>not linked</t>
         </is>
       </c>
       <c r="O65" s="3" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="N66" s="3" t="inlineStr">
         <is>
-          <t>not on ESPN</t>
+          <t>not linked</t>
         </is>
       </c>
       <c r="O66" s="3" t="inlineStr">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="N67" s="3" t="inlineStr">
         <is>
-          <t>not on ESPN</t>
+          <t>not linked</t>
         </is>
       </c>
       <c r="O67" s="3" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="N68" s="3" t="inlineStr">
         <is>
-          <t>not on ESPN</t>
+          <t>not linked</t>
         </is>
       </c>
       <c r="O68" s="3" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="N69" s="3" t="inlineStr">
         <is>
-          <t>not on ESPN</t>
+          <t>not linked</t>
         </is>
       </c>
       <c r="O69" s="3" t="inlineStr">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="N70" s="3" t="inlineStr">
         <is>
-          <t>not on ESPN</t>
+          <t>not linked</t>
         </is>
       </c>
       <c r="O70" s="3" t="inlineStr">
@@ -6601,7 +6601,7 @@
       </c>
       <c r="N71" s="3" t="inlineStr">
         <is>
-          <t>not on ESPN</t>
+          <t>not linked</t>
         </is>
       </c>
       <c r="O71" s="3" t="inlineStr">
@@ -7082,15 +7082,6 @@
           <t>gallaudet</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
         <v>24</v>
       </c>
@@ -7102,14 +7093,12 @@
           <t>glass_ios_vision</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>

</xml_diff>